<commit_message>
Sync form points from updated Clientes_catalogo sheet.
Confirm gid 1759250993 as the points source and tolerate sheet
cleanup (keep Contactos + catalog; Instrucciones optional).

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mantenimiento_wes/maestro/CONTACTOS_ENVIOS_ACTAS.xlsx
+++ b/mantenimiento_wes/maestro/CONTACTOS_ENVIOS_ACTAS.xlsx
@@ -24,231 +24,231 @@
     <t>Cliente</t>
   </si>
   <si>
+    <t>Máquina</t>
+  </si>
+  <si>
     <t>Máquina / sitio</t>
   </si>
   <si>
+    <t>Rol</t>
+  </si>
+  <si>
+    <t>AEB</t>
+  </si>
+  <si>
+    <t>Nombre</t>
+  </si>
+  <si>
+    <t>MATRIZ PRIMER PISO</t>
+  </si>
+  <si>
     <t>Este Excel es el registro de correos para el formulario de visita.</t>
   </si>
   <si>
-    <t>AEB</t>
-  </si>
-  <si>
-    <t>Máquina</t>
-  </si>
-  <si>
-    <t>MATRIZ PRIMER PISO</t>
+    <t>Cargo</t>
+  </si>
+  <si>
+    <t>MATRIZ RIEGO PLAZA</t>
+  </si>
+  <si>
+    <t>AGUNSA</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>DEPOSITO</t>
   </si>
   <si>
     <t>Columnas en la hoja Contactos:</t>
   </si>
   <si>
+    <t>MODULO ABC</t>
+  </si>
+  <si>
+    <t>Actualizado</t>
+  </si>
+  <si>
     <t xml:space="preserve">  • Cliente — ej. CORMUP</t>
   </si>
   <si>
-    <t>MATRIZ RIEGO PLAZA</t>
-  </si>
-  <si>
-    <t>Rol</t>
-  </si>
-  <si>
-    <t>AGUNSA</t>
+    <t>MODULO D</t>
   </si>
   <si>
     <t xml:space="preserve">  • Máquina — vacío si es el encargado GENERAL del cliente; o el colegio/sitio si es del PUNTO</t>
   </si>
   <si>
-    <t>DEPOSITO</t>
-  </si>
-  <si>
-    <t>Nombre</t>
+    <t>MODULO E</t>
   </si>
   <si>
     <t xml:space="preserve">  • Rol — general  |  punto</t>
   </si>
   <si>
-    <t>Cargo</t>
-  </si>
-  <si>
-    <t>MODULO ABC</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>MODULO D</t>
+    <t xml:space="preserve">INTERMODAL </t>
+  </si>
+  <si>
+    <t>COR. PUENTE</t>
   </si>
   <si>
     <t xml:space="preserve">  • Nombre / Cargo — opcional (inspector, director, etc.)</t>
   </si>
   <si>
-    <t>Actualizado</t>
+    <t>BOM</t>
+  </si>
+  <si>
+    <t>SAN IGNACIO 300</t>
   </si>
   <si>
     <t xml:space="preserve">  • Email — correo To (general) o CC (punto)</t>
   </si>
   <si>
-    <t>MODULO E</t>
+    <t>SAN IGNACIO 500</t>
+  </si>
+  <si>
+    <t>BUPA ANTOFGASTA</t>
   </si>
   <si>
     <t xml:space="preserve">  • Actualizado — fecha de última carga</t>
   </si>
   <si>
-    <t xml:space="preserve">INTERMODAL </t>
-  </si>
-  <si>
-    <t>COR. PUENTE</t>
-  </si>
-  <si>
-    <t>BOM</t>
+    <t>MEDIDOR PRINCIPAL SANITARIA</t>
+  </si>
+  <si>
+    <t>SALA DE BOMBA N°2</t>
   </si>
   <si>
     <t>Cómo se usa en el formulario:</t>
   </si>
   <si>
-    <t>SAN IGNACIO 300</t>
+    <t>SALA DE BOMBA SEXTO PISO</t>
+  </si>
+  <si>
+    <t>general</t>
   </si>
   <si>
     <t xml:space="preserve">  1) To = Email con Rol=general de ese Cliente</t>
   </si>
   <si>
-    <t>SAN IGNACIO 500</t>
+    <t>SALA DE BOMBAS PRINCIPAL</t>
   </si>
   <si>
     <t xml:space="preserve">  2) CC = Email con Rol=punto de ese Cliente + Máquina</t>
   </si>
   <si>
-    <t>BUPA ANTOFGASTA</t>
-  </si>
-  <si>
-    <t>MEDIDOR PRINCIPAL SANITARIA</t>
-  </si>
-  <si>
-    <t>general</t>
+    <t>CDUC</t>
+  </si>
+  <si>
+    <t>CALLE DE SERVICO</t>
   </si>
   <si>
     <t xml:space="preserve">  3) Al enviar una visita, el formulario actualiza también la hoja Contactos</t>
   </si>
   <si>
-    <t>SALA DE BOMBA N°2</t>
+    <t>CANCHAS DE TENIS</t>
+  </si>
+  <si>
+    <t>Rodrigo Toaboada</t>
   </si>
   <si>
     <t xml:space="preserve">     del Sheet de registro de fallas (misma lógica).</t>
   </si>
   <si>
+    <t>CLUB HOUSE</t>
+  </si>
+  <si>
     <t xml:space="preserve">  4) Aníbal (anibal.aoperaciones@wes.cl) siempre queda en CC además del punto.</t>
   </si>
   <si>
-    <t>SALA DE BOMBA SEXTO PISO</t>
-  </si>
-  <si>
-    <t>Rodrigo Toaboada</t>
-  </si>
-  <si>
-    <t>SALA DE BOMBAS PRINCIPAL</t>
+    <t>EQUITACION</t>
+  </si>
+  <si>
+    <t>RAIMUNDO TUPPER</t>
+  </si>
+  <si>
+    <t>Encargado general</t>
   </si>
   <si>
     <t>Podés editar esta planilla y pedirle al agente que la sincronice al formulario.</t>
   </si>
   <si>
-    <t>CDUC</t>
-  </si>
-  <si>
-    <t>CALLE DE SERVICO</t>
-  </si>
-  <si>
-    <t>Encargado general</t>
+    <t>COPEC</t>
+  </si>
+  <si>
+    <t>COSTANERA</t>
+  </si>
+  <si>
+    <t>ESTANQUE DE REUTILIZACION</t>
+  </si>
+  <si>
+    <t>rodrigo.taboada@cmpuentealto.cl</t>
   </si>
   <si>
     <t>Generado: 2026-08-13 18:41</t>
   </si>
   <si>
-    <t>CANCHAS DE TENIS</t>
-  </si>
-  <si>
-    <t>rodrigo.taboada@cmpuentealto.cl</t>
-  </si>
-  <si>
-    <t>CLUB HOUSE</t>
-  </si>
-  <si>
-    <t>EQUITACION</t>
-  </si>
-  <si>
-    <t>RAIMUNDO TUPPER</t>
-  </si>
-  <si>
-    <t>COPEC</t>
-  </si>
-  <si>
-    <t>COSTANERA</t>
+    <t>LAVADO AUTO SERVICIO NORTE</t>
+  </si>
+  <si>
+    <t>LAVADO AUTO SERVICIO SUR</t>
+  </si>
+  <si>
+    <t>LAVADO AUTOMATICO NORTE</t>
+  </si>
+  <si>
+    <t>LAVADO AUTOMATICO SUR</t>
+  </si>
+  <si>
+    <t>MATRIZ PRINCIPAL</t>
   </si>
   <si>
     <t>ESCUELA VILLA INDEPENDENCIA</t>
   </si>
   <si>
-    <t>ESTANQUE DE REUTILIZACION</t>
+    <t>OFICINA ADMIN</t>
+  </si>
+  <si>
+    <t>PRONTO BAÑO</t>
   </si>
   <si>
     <t>CC</t>
   </si>
   <si>
-    <t>LAVADO AUTO SERVICIO NORTE</t>
-  </si>
-  <si>
-    <t>LAVADO AUTO SERVICIO SUR</t>
-  </si>
-  <si>
-    <t>LAVADO AUTOMATICO NORTE</t>
+    <t>PRONTO TIENDA</t>
+  </si>
+  <si>
+    <t>RIEGO</t>
+  </si>
+  <si>
+    <t>COMPLEJO EDUCACIONAL CONSOLIDADA</t>
   </si>
   <si>
     <t>ESCUELA ANDES DEL SUR</t>
   </si>
   <si>
-    <t>LAVADO AUTOMATICO SUR</t>
-  </si>
-  <si>
-    <t>MATRIZ PRINCIPAL</t>
-  </si>
-  <si>
-    <t>OFICINA ADMIN</t>
-  </si>
-  <si>
-    <t>PRONTO BAÑO</t>
-  </si>
-  <si>
-    <t>PRONTO TIENDA</t>
-  </si>
-  <si>
-    <t>RIEGO</t>
+    <t>ESCUELA GABRIELA</t>
+  </si>
+  <si>
+    <t>ESCUELA JUAN MACKENNA</t>
+  </si>
+  <si>
+    <t>ESCUELA LOS ANDES</t>
+  </si>
+  <si>
+    <t>ESCUELA LUIS MATTE LARRAIN</t>
   </si>
   <si>
     <t>ESCUELA PADRE HURTADO</t>
   </si>
   <si>
-    <t>COMPLEJO EDUCACIONAL CONSOLIDADA</t>
-  </si>
-  <si>
-    <t>ESCUELA GABRIELA</t>
-  </si>
-  <si>
-    <t>ESCUELA JUAN MACKENNA</t>
-  </si>
-  <si>
-    <t>ESCUELA LOS ANDES</t>
+    <t>ESCULA NONATO COO</t>
+  </si>
+  <si>
+    <t>LICEO CHILOE</t>
   </si>
   <si>
     <t>LICEO MAIPO</t>
   </si>
   <si>
-    <t>ESCUELA LUIS MATTE LARRAIN</t>
-  </si>
-  <si>
-    <t>ESCULA NONATO COO</t>
-  </si>
-  <si>
-    <t>LICEO CHILOE</t>
-  </si>
-  <si>
     <t>CORMUP</t>
   </si>
   <si>
@@ -402,49 +402,145 @@
     <t>PIZZA HUT</t>
   </si>
   <si>
+    <t>SALA DE BOMBAS ESTANQUE SUR</t>
+  </si>
+  <si>
+    <t>MAM</t>
+  </si>
+  <si>
+    <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
+  </si>
+  <si>
+    <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
+  </si>
+  <si>
+    <t>PLACA BANCARIA</t>
+  </si>
+  <si>
+    <t>SALA DE BOMBAS FALABELLA</t>
+  </si>
+  <si>
+    <t>SALA DE BOMBAS RIPLEY</t>
+  </si>
+  <si>
+    <t>MAQ</t>
+  </si>
+  <si>
+    <t>ALIMENTACION DE BAÑOS</t>
+  </si>
+  <si>
+    <t>RED DE INCENDIO</t>
+  </si>
+  <si>
+    <t>NIDO</t>
+  </si>
+  <si>
+    <t>CONTROL NIDO</t>
+  </si>
+  <si>
+    <t>ELEMENTARY</t>
+  </si>
+  <si>
+    <t>ESTANQUE B</t>
+  </si>
+  <si>
+    <t>ESTANQUE C</t>
+  </si>
+  <si>
+    <t>HIGH SCHOOL</t>
+  </si>
+  <si>
+    <t>PISCINA</t>
+  </si>
+  <si>
+    <t>POZO PROFUNDO</t>
+  </si>
+  <si>
+    <t>TEATRO</t>
+  </si>
+  <si>
+    <t>PAK</t>
+  </si>
+  <si>
+    <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
+  </si>
+  <si>
+    <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
+  </si>
+  <si>
+    <t>ANDEN 3-4 RESTAURANTE</t>
+  </si>
+  <si>
+    <t>BAZAR GOURMET</t>
+  </si>
+  <si>
+    <t>DISTRITO DE LUJO</t>
+  </si>
+  <si>
+    <t>DL KENNEDY</t>
+  </si>
+  <si>
+    <t>LLENADO DE PILETA</t>
+  </si>
+  <si>
+    <t>PILETA CASCADA</t>
+  </si>
+  <si>
+    <t>SANDIA ANTIGUA</t>
+  </si>
+  <si>
+    <t>SANDIA NUEVA</t>
+  </si>
+  <si>
+    <t>PROVIDENCIA</t>
+  </si>
+  <si>
+    <t>CARMELA CARVAJAL</t>
+  </si>
+  <si>
+    <t>LASTARRIA</t>
+  </si>
+  <si>
+    <t>LICEO JUAN PABLO DUARTE</t>
+  </si>
+  <si>
+    <t>LICEO N°7</t>
+  </si>
+  <si>
+    <t>RENCA</t>
+  </si>
+  <si>
+    <t>ICCO</t>
+  </si>
+  <si>
+    <t>ICCP</t>
+  </si>
+  <si>
+    <t>ESCUELA LO VELEZQUEZ</t>
+  </si>
+  <si>
+    <t>GIMNASIO MUNICIPAL</t>
+  </si>
+  <si>
+    <t>PISCINA MUNICIPAL</t>
+  </si>
+  <si>
+    <t>UDD</t>
+  </si>
+  <si>
+    <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
+  </si>
+  <si>
+    <t>SALA DE BOMBAS HONDURAS</t>
+  </si>
+  <si>
     <t>dcampos.henriquez@cormup.cl</t>
   </si>
   <si>
-    <t>SALA DE BOMBAS ESTANQUE SUR</t>
-  </si>
-  <si>
-    <t>MAM</t>
-  </si>
-  <si>
-    <t>MATRIZ BOULEVARD PASILLO TECNICO</t>
-  </si>
-  <si>
-    <t>MATRIZ SALIDA DE EMERGENCIA PASILLO N°1 ARROW</t>
-  </si>
-  <si>
-    <t>PLACA BANCARIA</t>
-  </si>
-  <si>
-    <t>SALA DE BOMBAS FALABELLA</t>
-  </si>
-  <si>
-    <t>SALA DE BOMBAS RIPLEY</t>
-  </si>
-  <si>
-    <t>MAQ</t>
-  </si>
-  <si>
-    <t>ALIMENTACION DE BAÑOS</t>
-  </si>
-  <si>
     <t>MARIA PAZ FUENTEALBA</t>
   </si>
   <si>
-    <t>RED DE INCENDIO</t>
-  </si>
-  <si>
     <t>ADMINISTRADORA</t>
-  </si>
-  <si>
-    <t>NIDO</t>
-  </si>
-  <si>
-    <t>CONTROL NIDO</t>
   </si>
   <si>
     <r>
@@ -458,72 +554,6 @@
     </r>
   </si>
   <si>
-    <t>ELEMENTARY</t>
-  </si>
-  <si>
-    <t>ESTANQUE B</t>
-  </si>
-  <si>
-    <t>ESTANQUE C</t>
-  </si>
-  <si>
-    <t>HIGH SCHOOL</t>
-  </si>
-  <si>
-    <t>PISCINA</t>
-  </si>
-  <si>
-    <t>POZO PROFUNDO</t>
-  </si>
-  <si>
-    <t>TEATRO</t>
-  </si>
-  <si>
-    <t>PAK</t>
-  </si>
-  <si>
-    <t>ANDEN 3-4 LOCALES GASTRONOMICOS</t>
-  </si>
-  <si>
-    <t>ANDEN 3-4 MATRIZ PRINCIPAL</t>
-  </si>
-  <si>
-    <t>ANDEN 3-4 RESTAURANTE</t>
-  </si>
-  <si>
-    <t>BAZAR GOURMET</t>
-  </si>
-  <si>
-    <t>DISTRITO DE LUJO</t>
-  </si>
-  <si>
-    <t>DL KENNEDY</t>
-  </si>
-  <si>
-    <t>LLENADO DE PILETA</t>
-  </si>
-  <si>
-    <t>PILETA CASCADA</t>
-  </si>
-  <si>
-    <t>SANDIA ANTIGUA</t>
-  </si>
-  <si>
-    <t>SANDIA NUEVA</t>
-  </si>
-  <si>
-    <t>PROVIDENCIA</t>
-  </si>
-  <si>
-    <t>CARMELA CARVAJAL</t>
-  </si>
-  <si>
-    <t>LASTARRIA</t>
-  </si>
-  <si>
-    <t>LICEO JUAN PABLO DUARTE</t>
-  </si>
-  <si>
     <t>CLAUDIA FRUGOME</t>
   </si>
   <si>
@@ -539,36 +569,6 @@
       </rPr>
       <t>CFRUGONE.GONZALEZ@REDUCA.CL</t>
     </r>
-  </si>
-  <si>
-    <t>LICEO N°7</t>
-  </si>
-  <si>
-    <t>RENCA</t>
-  </si>
-  <si>
-    <t>ICCO</t>
-  </si>
-  <si>
-    <t>ICCP</t>
-  </si>
-  <si>
-    <t>ESCUELA LO VELEZQUEZ</t>
-  </si>
-  <si>
-    <t>GIMNASIO MUNICIPAL</t>
-  </si>
-  <si>
-    <t>PISCINA MUNICIPAL</t>
-  </si>
-  <si>
-    <t>UDD</t>
-  </si>
-  <si>
-    <t>SALA DE BOMBAS EDIFICIO ¨O¨</t>
-  </si>
-  <si>
-    <t>SALA DE BOMBAS HONDURAS</t>
   </si>
   <si>
     <t>C.E. VALLE HERMOSO</t>
@@ -1162,15 +1162,15 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="10.0"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10.0"/>
@@ -1262,12 +1262,6 @@
   <borders count="6">
     <border/>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFC5D5E6"/>
       </left>
@@ -1277,6 +1271,12 @@
       <top style="thin">
         <color rgb="FFC5D5E6"/>
       </top>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
     </border>
     <border>
       <left style="thin">
@@ -1317,28 +1317,28 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="2" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="2" fillId="2" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="4" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="5" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -1369,14 +1369,14 @@
     <xf borderId="5" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="5" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="5" fillId="0" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1409,10 +1409,10 @@
     <xf borderId="5" fillId="4" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1654,56 +1654,56 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="7" t="s">
+      <c r="B1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="8" t="s">
         <v>16</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="12" t="s">
         <v>35</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="G2" s="15"/>
     </row>
     <row r="3">
       <c r="A3" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D3" s="18"/>
       <c r="E3" s="14"/>
@@ -1712,13 +1712,13 @@
     </row>
     <row r="4">
       <c r="A4" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D4" s="18"/>
       <c r="E4" s="14"/>
@@ -1727,13 +1727,13 @@
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D5" s="18"/>
       <c r="E5" s="14"/>
@@ -1742,13 +1742,13 @@
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D6" s="18"/>
       <c r="E6" s="14"/>
@@ -1757,13 +1757,13 @@
     </row>
     <row r="7">
       <c r="A7" s="19" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D7" s="21"/>
       <c r="E7" s="21"/>
@@ -1772,13 +1772,13 @@
     </row>
     <row r="8">
       <c r="A8" s="19" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D8" s="21"/>
       <c r="E8" s="21"/>
@@ -1787,13 +1787,13 @@
     </row>
     <row r="9">
       <c r="A9" s="19" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B9" s="20" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D9" s="21"/>
       <c r="E9" s="21"/>
@@ -1802,13 +1802,13 @@
     </row>
     <row r="10">
       <c r="A10" s="19" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B10" s="20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D10" s="21"/>
       <c r="E10" s="21"/>
@@ -1817,13 +1817,13 @@
     </row>
     <row r="11">
       <c r="A11" s="19" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D11" s="21"/>
       <c r="E11" s="21"/>
@@ -1832,13 +1832,13 @@
     </row>
     <row r="12">
       <c r="A12" s="19" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D12" s="21"/>
       <c r="E12" s="21"/>
@@ -1847,13 +1847,13 @@
     </row>
     <row r="13">
       <c r="A13" s="19" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D13" s="21"/>
       <c r="E13" s="21"/>
@@ -1871,7 +1871,7 @@
       <c r="D14" s="23"/>
       <c r="E14" s="23"/>
       <c r="F14" s="23" t="s">
-        <v>128</v>
+        <v>172</v>
       </c>
       <c r="G14" s="25">
         <v>46251.64861111111</v>
@@ -1885,16 +1885,16 @@
         <v>79</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>138</v>
+        <v>173</v>
       </c>
       <c r="E15" s="27" t="s">
-        <v>140</v>
+        <v>174</v>
       </c>
       <c r="F15" s="28" t="s">
-        <v>143</v>
+        <v>175</v>
       </c>
       <c r="G15" s="22"/>
     </row>
@@ -1906,16 +1906,16 @@
         <v>80</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D16" s="27" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="E16" s="27" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="F16" s="28" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="G16" s="22"/>
     </row>
@@ -1927,7 +1927,7 @@
         <v>179</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D17" s="27" t="s">
         <v>180</v>
@@ -1948,7 +1948,7 @@
         <v>89</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D18" s="27" t="s">
         <v>183</v>
@@ -1969,7 +1969,7 @@
         <v>87</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D19" s="27" t="s">
         <v>186</v>
@@ -1990,7 +1990,7 @@
         <v>88</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D20" s="27" t="s">
         <v>188</v>
@@ -2011,7 +2011,7 @@
         <v>190</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D21" s="27" t="s">
         <v>191</v>
@@ -2032,7 +2032,7 @@
         <v>83</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D22" s="27" t="s">
         <v>194</v>
@@ -2053,7 +2053,7 @@
         <v>91</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D23" s="27" t="s">
         <v>197</v>
@@ -2074,7 +2074,7 @@
         <v>199</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D24" s="27" t="s">
         <v>200</v>
@@ -2095,7 +2095,7 @@
         <v>203</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D25" s="27" t="s">
         <v>204</v>
@@ -2116,7 +2116,7 @@
         <v>206</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D26" s="27" t="s">
         <v>207</v>
@@ -2137,7 +2137,7 @@
         <v>209</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D27" s="27" t="s">
         <v>210</v>
@@ -2156,7 +2156,7 @@
         <v>78</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="D28" s="27" t="s">
         <v>212</v>
@@ -2171,10 +2171,10 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C29" s="23" t="s">
         <v>35</v>
@@ -2192,10 +2192,10 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" s="20" t="s">
         <v>53</v>
-      </c>
-      <c r="B30" s="20" t="s">
-        <v>56</v>
       </c>
       <c r="C30" s="23" t="s">
         <v>35</v>
@@ -2213,10 +2213,10 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C31" s="23" t="s">
         <v>35</v>
@@ -2234,10 +2234,10 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C32" s="23" t="s">
         <v>35</v>
@@ -2255,10 +2255,10 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C33" s="23" t="s">
         <v>35</v>
@@ -2276,10 +2276,10 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C34" s="23" t="s">
         <v>35</v>
@@ -2297,10 +2297,10 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C35" s="23" t="s">
         <v>35</v>
@@ -2318,10 +2318,10 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C36" s="23" t="s">
         <v>35</v>
@@ -2339,10 +2339,10 @@
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B37" s="20" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C37" s="23" t="s">
         <v>35</v>
@@ -2360,10 +2360,10 @@
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C38" s="23" t="s">
         <v>35</v>
@@ -2381,10 +2381,10 @@
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B39" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C39" s="23" t="s">
         <v>35</v>
@@ -2402,10 +2402,10 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="20" t="s">
+        <v>138</v>
+      </c>
+      <c r="B40" s="20" t="s">
         <v>141</v>
-      </c>
-      <c r="B40" s="20" t="s">
-        <v>145</v>
       </c>
       <c r="C40" s="23" t="s">
         <v>35</v>
@@ -2423,10 +2423,10 @@
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="20" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C41" s="23" t="s">
         <v>35</v>
@@ -2444,10 +2444,10 @@
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="20" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C42" s="23" t="s">
         <v>35</v>
@@ -2465,10 +2465,10 @@
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="20" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B43" s="20" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C43" s="23" t="s">
         <v>35</v>
@@ -2486,10 +2486,10 @@
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="20" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C44" s="23" t="s">
         <v>35</v>
@@ -2507,10 +2507,10 @@
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="20" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B45" s="20" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C45" s="23" t="s">
         <v>35</v>
@@ -2528,10 +2528,10 @@
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="20" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B46" s="20" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C46" s="23" t="s">
         <v>35</v>
@@ -2549,10 +2549,10 @@
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="20" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B47" s="20" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C47" s="23" t="s">
         <v>35</v>
@@ -2631,7 +2631,7 @@
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B51" s="20"/>
       <c r="C51" s="23" t="s">
@@ -2650,10 +2650,10 @@
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C52" s="23" t="s">
         <v>223</v>
@@ -2671,10 +2671,10 @@
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="B53" s="20" t="s">
         <v>162</v>
-      </c>
-      <c r="B53" s="20" t="s">
-        <v>169</v>
       </c>
       <c r="C53" s="23" t="s">
         <v>223</v>
@@ -2692,10 +2692,10 @@
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C54" s="23" t="s">
         <v>223</v>
@@ -2713,10 +2713,10 @@
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="20" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B55" s="20" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C55" s="23" t="s">
         <v>223</v>
@@ -2881,7 +2881,7 @@
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="20" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B63" s="33"/>
       <c r="C63" s="23" t="s">
@@ -2917,10 +2917,10 @@
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="20" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B65" s="33" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="C65" s="23" t="s">
         <v>223</v>
@@ -2938,10 +2938,10 @@
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="20" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B66" s="33" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="C66" s="23" t="s">
         <v>35</v>
@@ -2959,10 +2959,10 @@
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="20" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B67" s="33" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="C67" s="23" t="s">
         <v>223</v>
@@ -2980,10 +2980,10 @@
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="20" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B68" s="33" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="C68" s="23" t="s">
         <v>35</v>
@@ -3001,10 +3001,10 @@
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="20" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B69" s="33" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="C69" s="23" t="s">
         <v>223</v>
@@ -3022,10 +3022,10 @@
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="20" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B70" s="33" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="C70" s="23" t="s">
         <v>35</v>
@@ -3043,10 +3043,10 @@
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="20" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B71" s="33" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="C71" s="23" t="s">
         <v>223</v>
@@ -3064,10 +3064,10 @@
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="20" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B72" s="33" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="C72" s="23" t="s">
         <v>223</v>
@@ -3130,7 +3130,7 @@
         <v>11</v>
       </c>
       <c r="B75" s="20" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C75" s="23" t="s">
         <v>35</v>
@@ -3151,7 +3151,7 @@
         <v>11</v>
       </c>
       <c r="B76" s="20" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C76" s="23" t="s">
         <v>35</v>
@@ -3172,7 +3172,7 @@
         <v>11</v>
       </c>
       <c r="B77" s="20" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C77" s="23" t="s">
         <v>35</v>
@@ -3211,10 +3211,10 @@
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="20" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B79" s="20" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C79" s="23" t="s">
         <v>35</v>
@@ -3232,10 +3232,10 @@
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="20" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B80" s="20" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C80" s="23" t="s">
         <v>35</v>
@@ -3253,10 +3253,10 @@
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="20" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B81" s="20" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C81" s="23" t="s">
         <v>35</v>
@@ -3274,10 +3274,10 @@
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="20" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B82" s="20" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C82" s="23" t="s">
         <v>35</v>
@@ -3295,7 +3295,7 @@
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="20" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B83" s="20" t="s">
         <v>279</v>
@@ -3316,10 +3316,10 @@
     </row>
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="20" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B84" s="20" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C84" s="23" t="s">
         <v>35</v>
@@ -3337,10 +3337,10 @@
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="20" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B85" s="20" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C85" s="23" t="s">
         <v>35</v>
@@ -3358,10 +3358,10 @@
     </row>
     <row r="86" ht="15.75" customHeight="1">
       <c r="A86" s="20" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B86" s="20" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C86" s="23" t="s">
         <v>35</v>
@@ -3379,10 +3379,10 @@
     </row>
     <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="20" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B87" s="20" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C87" s="23" t="s">
         <v>35</v>
@@ -3421,10 +3421,10 @@
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="20" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="B89" s="20" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="C89" s="23" t="s">
         <v>35</v>
@@ -3442,10 +3442,10 @@
     </row>
     <row r="90" ht="15.75" customHeight="1">
       <c r="A90" s="20" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="B90" s="20" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="C90" s="23" t="s">
         <v>35</v>
@@ -3857,7 +3857,7 @@
         <v>123</v>
       </c>
       <c r="B110" s="20" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C110" s="23" t="s">
         <v>223</v>
@@ -3878,7 +3878,7 @@
         <v>123</v>
       </c>
       <c r="B111" s="20" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C111" s="23" t="s">
         <v>303</v>
@@ -3915,10 +3915,10 @@
     </row>
     <row r="113" ht="15.75" customHeight="1">
       <c r="A113" s="35" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B113" s="35" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C113" s="23" t="s">
         <v>223</v>
@@ -3936,10 +3936,10 @@
     </row>
     <row r="114" ht="15.75" customHeight="1">
       <c r="A114" s="35" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B114" s="35" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C114" s="23" t="s">
         <v>311</v>
@@ -3951,10 +3951,10 @@
     </row>
     <row r="115" ht="15.75" customHeight="1">
       <c r="A115" s="35" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B115" s="35" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C115" s="23" t="s">
         <v>223</v>
@@ -3972,10 +3972,10 @@
     </row>
     <row r="116" ht="15.75" customHeight="1">
       <c r="A116" s="35" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B116" s="35" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C116" s="23" t="s">
         <v>311</v>
@@ -3987,7 +3987,7 @@
     </row>
     <row r="117" ht="15.75" customHeight="1">
       <c r="A117" s="35" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B117" s="35"/>
       <c r="C117" s="23" t="s">
@@ -4006,10 +4006,10 @@
     </row>
     <row r="118" ht="15.75" customHeight="1">
       <c r="A118" s="35" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B118" s="35" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C118" s="23" t="s">
         <v>223</v>
@@ -4027,7 +4027,7 @@
     </row>
     <row r="119" ht="15.75" customHeight="1">
       <c r="A119" s="35" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B119" s="11"/>
       <c r="C119" s="23" t="s">
@@ -4040,10 +4040,10 @@
     </row>
     <row r="120" ht="15.75" customHeight="1">
       <c r="A120" s="35" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B120" s="35" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C120" s="23" t="s">
         <v>223</v>
@@ -4061,7 +4061,7 @@
     </row>
     <row r="121" ht="15.75" customHeight="1">
       <c r="A121" s="35" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B121" s="11"/>
       <c r="C121" s="23" t="s">
@@ -4135,7 +4135,7 @@
     </row>
     <row r="125" ht="15.75" customHeight="1">
       <c r="A125" s="35" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B125" s="35"/>
       <c r="C125" s="23" t="s">
@@ -4154,10 +4154,10 @@
     </row>
     <row r="126" ht="15.75" customHeight="1">
       <c r="A126" s="35" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B126" s="35" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C126" s="23" t="s">
         <v>223</v>
@@ -4175,10 +4175,10 @@
     </row>
     <row r="127" ht="15.75" customHeight="1">
       <c r="A127" s="35" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B127" s="35" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C127" s="23" t="s">
         <v>223</v>
@@ -4196,10 +4196,10 @@
     </row>
     <row r="128" ht="15.75" customHeight="1">
       <c r="A128" s="35" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B128" s="35" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C128" s="23" t="s">
         <v>223</v>
@@ -4217,10 +4217,10 @@
     </row>
     <row r="129" ht="15.75" customHeight="1">
       <c r="A129" s="35" t="s">
+        <v>129</v>
+      </c>
+      <c r="B129" s="35" t="s">
         <v>130</v>
-      </c>
-      <c r="B129" s="35" t="s">
-        <v>131</v>
       </c>
       <c r="C129" s="23" t="s">
         <v>223</v>
@@ -4238,10 +4238,10 @@
     </row>
     <row r="130" ht="15.75" customHeight="1">
       <c r="A130" s="35" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B130" s="35" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C130" s="23" t="s">
         <v>223</v>
@@ -4259,7 +4259,7 @@
     </row>
     <row r="131" ht="15.75" customHeight="1">
       <c r="A131" s="35" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B131" s="35"/>
       <c r="C131" s="23" t="s">
@@ -4278,10 +4278,10 @@
     </row>
     <row r="132" ht="15.75" customHeight="1">
       <c r="A132" s="35" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B132" s="35" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C132" s="23" t="s">
         <v>223</v>
@@ -4299,10 +4299,10 @@
     </row>
     <row r="133" ht="15.75" customHeight="1">
       <c r="A133" s="35" t="s">
+        <v>135</v>
+      </c>
+      <c r="B133" s="35" t="s">
         <v>136</v>
-      </c>
-      <c r="B133" s="35" t="s">
-        <v>137</v>
       </c>
       <c r="C133" s="23" t="s">
         <v>223</v>
@@ -4320,7 +4320,7 @@
     </row>
     <row r="134" ht="15.75" customHeight="1">
       <c r="A134" s="35" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B134" s="35"/>
       <c r="C134" s="23" t="s">
@@ -4339,10 +4339,10 @@
     </row>
     <row r="135" ht="15.75" customHeight="1">
       <c r="A135" s="35" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B135" s="35" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C135" s="23" t="s">
         <v>223</v>
@@ -4360,10 +4360,10 @@
     </row>
     <row r="136" ht="15.75" customHeight="1">
       <c r="A136" s="35" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B136" s="35" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C136" s="23" t="s">
         <v>223</v>
@@ -4381,10 +4381,10 @@
     </row>
     <row r="137" ht="15.75" customHeight="1">
       <c r="A137" s="35" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B137" s="35" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C137" s="23" t="s">
         <v>223</v>
@@ -4402,10 +4402,10 @@
     </row>
     <row r="138" ht="15.75" customHeight="1">
       <c r="A138" s="35" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B138" s="35" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C138" s="23" t="s">
         <v>223</v>
@@ -4423,10 +4423,10 @@
     </row>
     <row r="139" ht="15.75" customHeight="1">
       <c r="A139" s="35" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B139" s="35" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C139" s="23" t="s">
         <v>223</v>
@@ -4444,10 +4444,10 @@
     </row>
     <row r="140" ht="15.75" customHeight="1">
       <c r="A140" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="B140" s="35" t="s">
         <v>151</v>
-      </c>
-      <c r="B140" s="35" t="s">
-        <v>155</v>
       </c>
       <c r="C140" s="23" t="s">
         <v>223</v>
@@ -4465,10 +4465,10 @@
     </row>
     <row r="141" ht="15.75" customHeight="1">
       <c r="A141" s="35" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B141" s="35" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C141" s="23" t="s">
         <v>223</v>
@@ -4486,10 +4486,10 @@
     </row>
     <row r="142" ht="15.75" customHeight="1">
       <c r="A142" s="35" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B142" s="35" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C142" s="23" t="s">
         <v>223</v>
@@ -4507,10 +4507,10 @@
     </row>
     <row r="143" ht="15.75" customHeight="1">
       <c r="A143" s="35" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B143" s="35" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C143" s="23" t="s">
         <v>223</v>
@@ -4528,10 +4528,10 @@
     </row>
     <row r="144" ht="15.75" customHeight="1">
       <c r="A144" s="35" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B144" s="35" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C144" s="23" t="s">
         <v>223</v>
@@ -11666,98 +11666,98 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3"/>
+      <c r="A2" s="5"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
-        <v>3</v>
+      <c r="A3" s="5" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3"/>
+      <c r="A4" s="5"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="s">
-        <v>7</v>
+      <c r="A5" s="5" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="s">
-        <v>8</v>
+      <c r="A6" s="5" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="s">
-        <v>12</v>
+      <c r="A7" s="5" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="s">
-        <v>15</v>
+      <c r="A8" s="5" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="s">
-        <v>20</v>
+      <c r="A9" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="s">
-        <v>22</v>
+      <c r="A10" s="5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="s">
-        <v>24</v>
+      <c r="A11" s="5" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3"/>
+      <c r="A12" s="5"/>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="s">
-        <v>28</v>
+      <c r="A13" s="5" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="s">
-        <v>30</v>
+      <c r="A14" s="5" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="s">
-        <v>32</v>
+      <c r="A15" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="s">
-        <v>36</v>
+      <c r="A16" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="s">
-        <v>38</v>
+      <c r="A17" s="5" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="s">
-        <v>39</v>
+      <c r="A18" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3"/>
+      <c r="A19" s="5"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="s">
-        <v>43</v>
+      <c r="A20" s="5" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="3"/>
+      <c r="A21" s="5"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="3" t="s">
-        <v>47</v>
+      <c r="A22" s="5" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1"/>
@@ -12759,575 +12759,575 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>2</v>
+      <c r="B1" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>6</v>
+      <c r="A2" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>9</v>
+      <c r="A3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>17</v>
+      <c r="B5" s="7" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>19</v>
+      <c r="B6" s="7" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="7" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="B30" s="5" t="s">
+      <c r="B31" s="7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B31" s="5" t="s">
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B33" s="7" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B32" s="5" t="s">
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B34" s="7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B38" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B36" s="5" t="s">
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B39" s="7" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B39" s="5" t="s">
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B40" s="7" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B40" s="5" t="s">
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B41" s="7" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="B42" s="7" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="5" t="s">
+      <c r="A43" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B43" s="7" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B44" s="7" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="5" t="s">
+      <c r="A45" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="7" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="5" t="s">
+      <c r="A46" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="7" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="5" t="s">
+      <c r="A47" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B47" s="7" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="5" t="s">
+      <c r="A48" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="B48" s="7" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="5" t="s">
+      <c r="A49" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="7" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="5" t="s">
+      <c r="A50" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="B50" s="7" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="5" t="s">
+      <c r="A51" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B51" s="5" t="s">
+      <c r="B51" s="7" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="5" t="s">
+      <c r="A52" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B52" s="7" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="5" t="s">
+      <c r="A53" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="B53" s="7" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="5" t="s">
+      <c r="A54" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B54" s="5" t="s">
+      <c r="B54" s="7" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="5" t="s">
+      <c r="A55" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="B55" s="7" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="5" t="s">
+      <c r="A56" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B56" s="5" t="s">
+      <c r="B56" s="7" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="5" t="s">
+      <c r="A57" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B57" s="5" t="s">
+      <c r="B57" s="7" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="5" t="s">
+      <c r="A58" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="B58" s="7" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="5" t="s">
+      <c r="A59" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B59" s="5" t="s">
+      <c r="B59" s="7" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="5" t="s">
+      <c r="A60" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="B60" s="7" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="5" t="s">
+      <c r="A61" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B61" s="5" t="s">
+      <c r="B61" s="7" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="5" t="s">
+      <c r="A62" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B62" s="5" t="s">
+      <c r="B62" s="7" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="5" t="s">
+      <c r="A63" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B63" s="5" t="s">
+      <c r="B63" s="7" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="A64" s="5" t="s">
+      <c r="A64" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="B64" s="7" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="5" t="s">
+      <c r="A65" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B65" s="5" t="s">
+      <c r="B65" s="7" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="5" t="s">
+      <c r="A66" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B66" s="5" t="s">
+      <c r="B66" s="7" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="5" t="s">
+      <c r="A67" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B67" s="5" t="s">
+      <c r="B67" s="7" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
-      <c r="A68" s="5" t="s">
+      <c r="A68" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B68" s="5" t="s">
+      <c r="B68" s="7" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="5" t="s">
+      <c r="A69" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="B69" s="7" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
-      <c r="A70" s="5" t="s">
+      <c r="A70" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B70" s="5" t="s">
+      <c r="B70" s="7" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
-      <c r="A71" s="5" t="s">
+      <c r="A71" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B71" s="5" t="s">
+      <c r="B71" s="7" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="72" ht="15.75" customHeight="1">
-      <c r="A72" s="5" t="s">
+      <c r="A72" s="7" t="s">
         <v>103</v>
       </c>
       <c r="B72" s="9" t="s">
@@ -13335,395 +13335,395 @@
       </c>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="5" t="s">
+      <c r="A73" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="B73" s="5" t="s">
+      <c r="B73" s="7" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="A74" s="5" t="s">
+      <c r="A74" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="B74" s="5" t="s">
+      <c r="B74" s="7" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="5" t="s">
+      <c r="A75" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="B75" s="5" t="s">
+      <c r="B75" s="7" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="5" t="s">
+      <c r="A76" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="B76" s="5" t="s">
+      <c r="B76" s="7" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="A77" s="5" t="s">
+      <c r="A77" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="B77" s="5" t="s">
+      <c r="B77" s="7" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="5" t="s">
+      <c r="A78" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="B78" s="5" t="s">
+      <c r="B78" s="7" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="79" ht="15.75" customHeight="1">
-      <c r="A79" s="5" t="s">
+      <c r="A79" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="B79" s="5" t="s">
+      <c r="B79" s="7" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="80" ht="15.75" customHeight="1">
-      <c r="A80" s="5" t="s">
+      <c r="A80" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B80" s="5" t="s">
+      <c r="B80" s="7" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="81" ht="15.75" customHeight="1">
-      <c r="A81" s="5" t="s">
+      <c r="A81" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B81" s="5" t="s">
+      <c r="B81" s="7" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="82" ht="15.75" customHeight="1">
-      <c r="A82" s="5" t="s">
+      <c r="A82" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B82" s="5" t="s">
+      <c r="B82" s="7" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="83" ht="15.75" customHeight="1">
-      <c r="A83" s="5" t="s">
+      <c r="A83" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B83" s="5" t="s">
+      <c r="B83" s="7" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="84" ht="15.75" customHeight="1">
-      <c r="A84" s="5" t="s">
+      <c r="A84" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="B84" s="5" t="s">
+      <c r="B84" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="85" ht="15.75" customHeight="1">
+      <c r="A85" s="7" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="85" ht="15.75" customHeight="1">
-      <c r="A85" s="5" t="s">
+      <c r="B85" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="B85" s="5" t="s">
+    </row>
+    <row r="86" ht="15.75" customHeight="1">
+      <c r="A86" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B86" s="7" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="86" ht="15.75" customHeight="1">
-      <c r="A86" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="B86" s="5" t="s">
+    <row r="87" ht="15.75" customHeight="1">
+      <c r="A87" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B87" s="7" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="87" ht="15.75" customHeight="1">
-      <c r="A87" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="B87" s="5" t="s">
+    <row r="88" ht="15.75" customHeight="1">
+      <c r="A88" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B88" s="7" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="88" ht="15.75" customHeight="1">
-      <c r="A88" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="B88" s="5" t="s">
+    <row r="89" ht="15.75" customHeight="1">
+      <c r="A89" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B89" s="7" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="89" ht="15.75" customHeight="1">
-      <c r="A89" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="B89" s="5" t="s">
+    <row r="90" ht="15.75" customHeight="1">
+      <c r="A90" s="7" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="90" ht="15.75" customHeight="1">
-      <c r="A90" s="5" t="s">
+      <c r="B90" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="B90" s="5" t="s">
+    </row>
+    <row r="91" ht="15.75" customHeight="1">
+      <c r="A91" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B91" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="92" ht="15.75" customHeight="1">
+      <c r="A92" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B92" s="7" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="91" ht="15.75" customHeight="1">
-      <c r="A91" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="B91" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="92" ht="15.75" customHeight="1">
-      <c r="A92" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="B92" s="5" t="s">
+    <row r="93" ht="15.75" customHeight="1">
+      <c r="A93" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B93" s="7" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="93" ht="15.75" customHeight="1">
-      <c r="A93" s="5" t="s">
+    <row r="94" ht="15.75" customHeight="1">
+      <c r="A94" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B94" s="7" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="95" ht="15.75" customHeight="1">
+      <c r="A95" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B95" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="B93" s="5" t="s">
+    </row>
+    <row r="96" ht="15.75" customHeight="1">
+      <c r="A96" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B96" s="7" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="94" ht="15.75" customHeight="1">
-      <c r="A94" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="B94" s="5" t="s">
+    <row r="97" ht="15.75" customHeight="1">
+      <c r="A97" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B97" s="7" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="98" ht="15.75" customHeight="1">
+      <c r="A98" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B98" s="7" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="95" ht="15.75" customHeight="1">
-      <c r="A95" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="B95" s="5" t="s">
+    <row r="99" ht="15.75" customHeight="1">
+      <c r="A99" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B99" s="7" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="96" ht="15.75" customHeight="1">
-      <c r="A96" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="B96" s="5" t="s">
+    <row r="100" ht="15.75" customHeight="1">
+      <c r="A100" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B100" s="7" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="97" ht="15.75" customHeight="1">
-      <c r="A97" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="B97" s="5" t="s">
+    <row r="101" ht="15.75" customHeight="1">
+      <c r="A101" s="7" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="98" ht="15.75" customHeight="1">
-      <c r="A98" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="B98" s="5" t="s">
+      <c r="B101" s="7" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="99" ht="15.75" customHeight="1">
-      <c r="A99" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="B99" s="5" t="s">
+    <row r="102" ht="15.75" customHeight="1">
+      <c r="A102" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B102" s="7" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="100" ht="15.75" customHeight="1">
-      <c r="A100" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="B100" s="5" t="s">
+    <row r="103" ht="15.75" customHeight="1">
+      <c r="A103" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B103" s="7" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="101" ht="15.75" customHeight="1">
-      <c r="A101" s="5" t="s">
+    <row r="104" ht="15.75" customHeight="1">
+      <c r="A104" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B104" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="B101" s="5" t="s">
+    </row>
+    <row r="105" ht="15.75" customHeight="1">
+      <c r="A105" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B105" s="7" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="102" ht="15.75" customHeight="1">
-      <c r="A102" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="B102" s="5" t="s">
+    <row r="106" ht="15.75" customHeight="1">
+      <c r="A106" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B106" s="7" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="103" ht="15.75" customHeight="1">
-      <c r="A103" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="B103" s="5" t="s">
+    <row r="107" ht="15.75" customHeight="1">
+      <c r="A107" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B107" s="7" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="104" ht="15.75" customHeight="1">
-      <c r="A104" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="B104" s="5" t="s">
+    <row r="108" ht="15.75" customHeight="1">
+      <c r="A108" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B108" s="7" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="105" ht="15.75" customHeight="1">
-      <c r="A105" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="B105" s="5" t="s">
+    <row r="109" ht="15.75" customHeight="1">
+      <c r="A109" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B109" s="7" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="106" ht="15.75" customHeight="1">
-      <c r="A106" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="B106" s="5" t="s">
+    <row r="110" ht="15.75" customHeight="1">
+      <c r="A110" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B110" s="7" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="107" ht="15.75" customHeight="1">
-      <c r="A107" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="B107" s="5" t="s">
+    <row r="111" ht="15.75" customHeight="1">
+      <c r="A111" s="7" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="108" ht="15.75" customHeight="1">
-      <c r="A108" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="B108" s="5" t="s">
+      <c r="B111" s="7" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="109" ht="15.75" customHeight="1">
-      <c r="A109" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="B109" s="5" t="s">
+    <row r="112" ht="15.75" customHeight="1">
+      <c r="A112" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B112" s="7" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="110" ht="15.75" customHeight="1">
-      <c r="A110" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="B110" s="5" t="s">
+    <row r="113" ht="15.75" customHeight="1">
+      <c r="A113" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B113" s="7" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="111" ht="15.75" customHeight="1">
-      <c r="A111" s="5" t="s">
+    <row r="114" ht="15.75" customHeight="1">
+      <c r="A114" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B114" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="B111" s="5" t="s">
+    </row>
+    <row r="115" ht="15.75" customHeight="1">
+      <c r="A115" s="7" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="112" ht="15.75" customHeight="1">
-      <c r="A112" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="B112" s="5" t="s">
+      <c r="B115" s="9" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="113" ht="15.75" customHeight="1">
-      <c r="A113" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="B113" s="5" t="s">
+    <row r="116" ht="15.75" customHeight="1">
+      <c r="A116" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="B116" s="9" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="114" ht="15.75" customHeight="1">
-      <c r="A114" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="B114" s="5" t="s">
+    <row r="117" ht="15.75" customHeight="1">
+      <c r="A117" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="B117" s="9" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="118" ht="15.75" customHeight="1">
+      <c r="A118" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="B118" s="9" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="119" ht="15.75" customHeight="1">
+      <c r="A119" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="B119" s="9" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="120" ht="15.75" customHeight="1">
+      <c r="A120" s="7" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="115" ht="15.75" customHeight="1">
-      <c r="A115" s="5" t="s">
+      <c r="B120" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="B115" s="9" t="s">
+    </row>
+    <row r="121" ht="15.75" customHeight="1">
+      <c r="A121" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B121" s="7" t="s">
         <v>171</v>
-      </c>
-    </row>
-    <row r="116" ht="15.75" customHeight="1">
-      <c r="A116" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B116" s="9" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="117" ht="15.75" customHeight="1">
-      <c r="A117" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B117" s="9" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="118" ht="15.75" customHeight="1">
-      <c r="A118" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B118" s="9" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="119" ht="15.75" customHeight="1">
-      <c r="A119" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="B119" s="9" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="120" ht="15.75" customHeight="1">
-      <c r="A120" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="B120" s="5" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="121" ht="15.75" customHeight="1">
-      <c r="A121" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="B121" s="5" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="122" ht="15.75" customHeight="1"/>

</xml_diff>